<commit_message>
Inicialización del backend y modelado de base de datos. - Creación de docker-compose.yml y Dockerfile - Conexión a base de datos gymflow (puerto 3350) - Creado en entidades
</commit_message>
<xml_diff>
--- a/GYMFLOW.xlsx
+++ b/GYMFLOW.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\abolt\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kiladew/DAW 2/PROYECTO INTERMODULAR/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9959339C-D125-4C23-B8FF-8197AB7E1190}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A3F9BE1-B95E-AC44-8DE4-5C6C5C191A23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="3" xr2:uid="{7169C136-EA6B-49E2-A7AA-B657C616E084}"/>
+    <workbookView xWindow="55000" yWindow="-7540" windowWidth="25600" windowHeight="28200" xr2:uid="{7169C136-EA6B-49E2-A7AA-B657C616E084}"/>
   </bookViews>
   <sheets>
     <sheet name="Grupos Musculares" sheetId="1" r:id="rId1"/>
@@ -42,9 +42,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="268" uniqueCount="157">
   <si>
-    <t>imagen</t>
-  </si>
-  <si>
     <t xml:space="preserve">Pecho </t>
   </si>
   <si>
@@ -511,6 +508,9 @@
   </si>
   <si>
     <t>stabilizer</t>
+  </si>
+  <si>
+    <t>image</t>
   </si>
 </sst>
 </file>
@@ -562,13 +562,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -904,80 +904,80 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{86D4A9B7-58CB-45E2-AB47-F96ECF111482}">
   <dimension ref="A1:C8"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" s="2" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C3" s="2"/>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C4" s="2"/>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2"/>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C6" s="2"/>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C7" s="2"/>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C8" s="2"/>
     </row>
@@ -992,32 +992,32 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BC5C106-8B90-4140-81B0-CA275B099F15}">
   <dimension ref="A1:C30"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.5" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.83203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -1025,10 +1025,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -1036,10 +1036,10 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -1047,10 +1047,10 @@
         <v>2</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -1058,10 +1058,10 @@
         <v>2</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -1069,10 +1069,10 @@
         <v>2</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -1080,10 +1080,10 @@
         <v>2</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -1091,10 +1091,10 @@
         <v>2</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -1102,10 +1102,10 @@
         <v>2</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -1113,10 +1113,10 @@
         <v>2</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -1124,10 +1124,10 @@
         <v>3</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -1135,10 +1135,10 @@
         <v>3</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -1146,10 +1146,10 @@
         <v>3</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -1157,10 +1157,10 @@
         <v>3</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>111</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -1168,10 +1168,10 @@
         <v>3</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>15</v>
       </c>
@@ -1179,10 +1179,10 @@
         <v>3</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -1190,10 +1190,10 @@
         <v>3</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -1201,10 +1201,10 @@
         <v>3</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -1212,10 +1212,10 @@
         <v>3</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -1223,10 +1223,10 @@
         <v>4</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -1234,10 +1234,10 @@
         <v>4</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -1245,10 +1245,10 @@
         <v>4</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -1256,10 +1256,10 @@
         <v>5</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -1267,10 +1267,10 @@
         <v>5</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -1278,10 +1278,10 @@
         <v>5</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -1289,10 +1289,10 @@
         <v>5</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -1300,10 +1300,10 @@
         <v>6</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -1311,10 +1311,10 @@
         <v>6</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>28</v>
       </c>
@@ -1322,7 +1322,7 @@
         <v>6</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>
@@ -1336,535 +1336,535 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{56917D66-D4F5-4776-89AD-3AE858058BAA}">
   <dimension ref="A1:C48"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="22.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="16.140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.42578125" customWidth="1"/>
-    <col min="6" max="6" width="23.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="31.28515625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.1640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.1640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.5" customWidth="1"/>
+    <col min="6" max="6" width="23.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="31.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>84</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>85</v>
-      </c>
       <c r="B2" s="2" t="s">
+        <v>50</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C4" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="C5" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>4</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C6" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>5</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C7" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>6</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>7</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C9" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>8</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C10" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>9</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C11" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>10</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C12" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>11</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>12</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C14" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>13</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C15" s="2">
         <v>2</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>14</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C16" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>15</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C17" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>16</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C18" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>17</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C19" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>18</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C20" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>19</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C21" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>20</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C22" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>21</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C23" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>22</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C24" s="2">
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>23</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C25" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>24</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C26" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>25</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C27" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>26</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C28" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>27</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C29" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>28</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C30" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
         <v>29</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C31" s="2">
         <v>4</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>30</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C32" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>31</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C33" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>32</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C34" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>33</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C35" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>34</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C36" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>35</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C37" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>36</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C38" s="2">
         <v>5</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>37</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C39" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>38</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C40" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>39</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C41" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>40</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C42" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>41</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C43" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>42</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C44" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>43</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C45" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>44</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C46" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>45</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C47" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>46</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C48" s="2">
         <v>6</v>
@@ -1881,32 +1881,32 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70B0D9F1-6646-4C30-AECB-5F69DB69F4A6}">
   <dimension ref="A1:C111"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>92</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -1914,10 +1914,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>1</v>
       </c>
@@ -1925,10 +1925,10 @@
         <v>23</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>1</v>
       </c>
@@ -1936,10 +1936,10 @@
         <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>2</v>
       </c>
@@ -1947,10 +1947,10 @@
         <v>1</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>2</v>
       </c>
@@ -1958,10 +1958,10 @@
         <v>20</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>3</v>
       </c>
@@ -1969,10 +1969,10 @@
         <v>1</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>4</v>
       </c>
@@ -1980,10 +1980,10 @@
         <v>1</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>5</v>
       </c>
@@ -1991,10 +1991,10 @@
         <v>1</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>5</v>
       </c>
@@ -2002,10 +2002,10 @@
         <v>3</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>6</v>
       </c>
@@ -2013,10 +2013,10 @@
         <v>1</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>6</v>
       </c>
@@ -2024,10 +2024,10 @@
         <v>23</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>7</v>
       </c>
@@ -2035,10 +2035,10 @@
         <v>1</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>7</v>
       </c>
@@ -2046,10 +2046,10 @@
         <v>23</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>8</v>
       </c>
@@ -2057,10 +2057,10 @@
         <v>5</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>8</v>
       </c>
@@ -2068,10 +2068,10 @@
         <v>15</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>8</v>
       </c>
@@ -2079,10 +2079,10 @@
         <v>14</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>9</v>
       </c>
@@ -2090,10 +2090,10 @@
         <v>3</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>9</v>
       </c>
@@ -2101,10 +2101,10 @@
         <v>9</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>9</v>
       </c>
@@ -2112,10 +2112,10 @@
         <v>4</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>9</v>
       </c>
@@ -2123,10 +2123,10 @@
         <v>22</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>10</v>
       </c>
@@ -2134,10 +2134,10 @@
         <v>3</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>10</v>
       </c>
@@ -2145,10 +2145,10 @@
         <v>9</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>10</v>
       </c>
@@ -2156,10 +2156,10 @@
         <v>4</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>10</v>
       </c>
@@ -2167,10 +2167,10 @@
         <v>22</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>11</v>
       </c>
@@ -2178,10 +2178,10 @@
         <v>3</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>11</v>
       </c>
@@ -2189,10 +2189,10 @@
         <v>6</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>11</v>
       </c>
@@ -2200,10 +2200,10 @@
         <v>22</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>11</v>
       </c>
@@ -2211,10 +2211,10 @@
         <v>24</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
         <v>12</v>
       </c>
@@ -2222,10 +2222,10 @@
         <v>3</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>12</v>
       </c>
@@ -2233,10 +2233,10 @@
         <v>6</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>12</v>
       </c>
@@ -2244,10 +2244,10 @@
         <v>22</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>13</v>
       </c>
@@ -2255,10 +2255,10 @@
         <v>4</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>13</v>
       </c>
@@ -2266,10 +2266,10 @@
         <v>5</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>14</v>
       </c>
@@ -2277,10 +2277,10 @@
         <v>10</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>14</v>
       </c>
@@ -2288,10 +2288,10 @@
         <v>15</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>14</v>
       </c>
@@ -2299,10 +2299,10 @@
         <v>14</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>14</v>
       </c>
@@ -2310,10 +2310,10 @@
         <v>11</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>14</v>
       </c>
@@ -2321,10 +2321,10 @@
         <v>16</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>15</v>
       </c>
@@ -2332,10 +2332,10 @@
         <v>10</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>16</v>
       </c>
@@ -2343,10 +2343,10 @@
         <v>14</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>17</v>
       </c>
@@ -2354,10 +2354,10 @@
         <v>15</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>17</v>
       </c>
@@ -2365,10 +2365,10 @@
         <v>14</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>17</v>
       </c>
@@ -2376,10 +2376,10 @@
         <v>16</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>18</v>
       </c>
@@ -2387,10 +2387,10 @@
         <v>15</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>18</v>
       </c>
@@ -2398,10 +2398,10 @@
         <v>16</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>19</v>
       </c>
@@ -2409,10 +2409,10 @@
         <v>10</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>19</v>
       </c>
@@ -2420,10 +2420,10 @@
         <v>15</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>19</v>
       </c>
@@ -2431,10 +2431,10 @@
         <v>14</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>19</v>
       </c>
@@ -2442,10 +2442,10 @@
         <v>16</v>
       </c>
       <c r="C51" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>20</v>
       </c>
@@ -2453,10 +2453,10 @@
         <v>10</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
         <v>20</v>
       </c>
@@ -2464,10 +2464,10 @@
         <v>15</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
         <v>20</v>
       </c>
@@ -2475,10 +2475,10 @@
         <v>14</v>
       </c>
       <c r="C54" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
         <v>21</v>
       </c>
@@ -2486,10 +2486,10 @@
         <v>10</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
         <v>21</v>
       </c>
@@ -2497,10 +2497,10 @@
         <v>15</v>
       </c>
       <c r="C56" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
         <v>21</v>
       </c>
@@ -2508,10 +2508,10 @@
         <v>14</v>
       </c>
       <c r="C57" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
         <v>22</v>
       </c>
@@ -2519,10 +2519,10 @@
         <v>10</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
         <v>22</v>
       </c>
@@ -2530,10 +2530,10 @@
         <v>15</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
         <v>22</v>
       </c>
@@ -2541,10 +2541,10 @@
         <v>14</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
         <v>22</v>
       </c>
@@ -2552,10 +2552,10 @@
         <v>16</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A62" s="2">
         <v>23</v>
       </c>
@@ -2563,10 +2563,10 @@
         <v>19</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A63" s="2">
         <v>23</v>
       </c>
@@ -2574,10 +2574,10 @@
         <v>20</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A64" s="2">
         <v>23</v>
       </c>
@@ -2585,10 +2585,10 @@
         <v>23</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A65" s="2">
         <v>24</v>
       </c>
@@ -2596,10 +2596,10 @@
         <v>19</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A66" s="2">
         <v>24</v>
       </c>
@@ -2607,10 +2607,10 @@
         <v>20</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A67" s="2">
         <v>24</v>
       </c>
@@ -2618,10 +2618,10 @@
         <v>23</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A68" s="2">
         <v>25</v>
       </c>
@@ -2629,10 +2629,10 @@
         <v>19</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A69" s="1">
         <v>26</v>
       </c>
@@ -2640,10 +2640,10 @@
         <v>20</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="70" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A70" s="1">
         <v>26</v>
       </c>
@@ -2651,10 +2651,10 @@
         <v>4</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A71" s="1">
         <v>27</v>
       </c>
@@ -2662,10 +2662,10 @@
         <v>20</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="72" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A72" s="1">
         <v>27</v>
       </c>
@@ -2673,10 +2673,10 @@
         <v>4</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="73" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A73" s="1">
         <v>27</v>
       </c>
@@ -2684,10 +2684,10 @@
         <v>22</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="74" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A74" s="1">
         <v>28</v>
       </c>
@@ -2695,10 +2695,10 @@
         <v>19</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="75" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A75" s="1">
         <v>29</v>
       </c>
@@ -2706,10 +2706,10 @@
         <v>21</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="76" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A76" s="1">
         <v>29</v>
       </c>
@@ -2717,10 +2717,10 @@
         <v>4</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="77" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A77" s="1">
         <v>30</v>
       </c>
@@ -2728,10 +2728,10 @@
         <v>22</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="78" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A78" s="1">
         <v>30</v>
       </c>
@@ -2739,10 +2739,10 @@
         <v>24</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A79" s="1">
         <v>30</v>
       </c>
@@ -2750,10 +2750,10 @@
         <v>25</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="80" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A80" s="1">
         <v>31</v>
       </c>
@@ -2761,10 +2761,10 @@
         <v>22</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="81" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A81" s="1">
         <v>31</v>
       </c>
@@ -2772,10 +2772,10 @@
         <v>24</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="82" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A82" s="1">
         <v>32</v>
       </c>
@@ -2783,10 +2783,10 @@
         <v>25</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A83" s="1">
         <v>32</v>
       </c>
@@ -2794,10 +2794,10 @@
         <v>24</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" s="1">
         <v>32</v>
       </c>
@@ -2805,10 +2805,10 @@
         <v>22</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="85" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A85" s="1">
         <v>33</v>
       </c>
@@ -2816,10 +2816,10 @@
         <v>23</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="86" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A86" s="1">
         <v>34</v>
       </c>
@@ -2827,10 +2827,10 @@
         <v>23</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="87" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A87" s="1">
         <v>35</v>
       </c>
@@ -2838,10 +2838,10 @@
         <v>23</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A88" s="1">
         <v>35</v>
       </c>
@@ -2849,10 +2849,10 @@
         <v>22</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A89" s="1">
         <v>36</v>
       </c>
@@ -2860,10 +2860,10 @@
         <v>23</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A90" s="1">
         <v>36</v>
       </c>
@@ -2871,10 +2871,10 @@
         <v>22</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A91" s="1">
         <v>37</v>
       </c>
@@ -2882,10 +2882,10 @@
         <v>28</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="92" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A92" s="1">
         <v>37</v>
       </c>
@@ -2893,10 +2893,10 @@
         <v>26</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A93" s="1">
         <v>37</v>
       </c>
@@ -2904,10 +2904,10 @@
         <v>27</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A94" s="1">
         <v>38</v>
       </c>
@@ -2915,10 +2915,10 @@
         <v>28</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A95" s="1">
         <v>38</v>
       </c>
@@ -2926,10 +2926,10 @@
         <v>26</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A96" s="1">
         <v>39</v>
       </c>
@@ -2937,10 +2937,10 @@
         <v>5</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A97" s="1">
         <v>39</v>
       </c>
@@ -2948,10 +2948,10 @@
         <v>28</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A98" s="1">
         <v>40</v>
       </c>
@@ -2959,10 +2959,10 @@
         <v>26</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A99" s="1">
         <v>40</v>
       </c>
@@ -2970,10 +2970,10 @@
         <v>27</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A100" s="1">
         <v>41</v>
       </c>
@@ -2981,10 +2981,10 @@
         <v>27</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A101" s="1">
         <v>41</v>
       </c>
@@ -2992,10 +2992,10 @@
         <v>28</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A102" s="1">
         <v>42</v>
       </c>
@@ -3003,10 +3003,10 @@
         <v>28</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A103" s="1">
         <v>42</v>
       </c>
@@ -3014,10 +3014,10 @@
         <v>27</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A104" s="1">
         <v>43</v>
       </c>
@@ -3025,10 +3025,10 @@
         <v>15</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A105" s="1">
         <v>43</v>
       </c>
@@ -3036,10 +3036,10 @@
         <v>5</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A106" s="1">
         <v>44</v>
       </c>
@@ -3047,10 +3047,10 @@
         <v>5</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" s="1">
         <v>44</v>
       </c>
@@ -3058,10 +3058,10 @@
         <v>15</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A108" s="1">
         <v>45</v>
       </c>
@@ -3069,10 +3069,10 @@
         <v>27</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A109" s="1">
         <v>45</v>
       </c>
@@ -3080,10 +3080,10 @@
         <v>26</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A110" s="1">
         <v>46</v>
       </c>
@@ -3091,10 +3091,10 @@
         <v>26</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>94</v>
-      </c>
-    </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A111" s="1">
         <v>46</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>28</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>
@@ -3116,30 +3116,30 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{75413422-EA62-43A9-8B45-9FBECA777D49}">
   <dimension ref="A1:I61"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="3" max="3" width="33.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="33.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>96</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-    </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>97</v>
-      </c>
       <c r="B2" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" s="2">
         <v>1</v>
       </c>
@@ -3147,10 +3147,10 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4" s="2">
         <v>2</v>
       </c>
@@ -3158,10 +3158,10 @@
         <v>2</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" s="2">
         <v>3</v>
       </c>
@@ -3169,10 +3169,10 @@
         <v>3</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" s="2">
         <v>4</v>
       </c>
@@ -3180,10 +3180,10 @@
         <v>3</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" s="2">
         <v>5</v>
       </c>
@@ -3191,10 +3191,10 @@
         <v>7</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="2">
         <v>6</v>
       </c>
@@ -3202,10 +3202,10 @@
         <v>8</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="2">
         <v>7</v>
       </c>
@@ -3213,10 +3213,10 @@
         <v>8</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" s="2">
         <v>8</v>
       </c>
@@ -3224,10 +3224,10 @@
         <v>9</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" s="2">
         <v>9</v>
       </c>
@@ -3235,10 +3235,10 @@
         <v>10</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" s="2">
         <v>10</v>
       </c>
@@ -3246,10 +3246,10 @@
         <v>10</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" s="2">
         <v>11</v>
       </c>
@@ -3257,10 +3257,10 @@
         <v>11</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" s="2">
         <v>12</v>
       </c>
@@ -3268,10 +3268,10 @@
         <v>12</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" s="2">
         <v>13</v>
       </c>
@@ -3279,10 +3279,10 @@
         <v>13</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" s="2">
         <v>14</v>
       </c>
@@ -3290,10 +3290,10 @@
         <v>14</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A17" s="2">
         <v>15</v>
       </c>
@@ -3301,10 +3301,10 @@
         <v>15</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18" s="2">
         <v>16</v>
       </c>
@@ -3312,10 +3312,10 @@
         <v>16</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" s="2">
         <v>17</v>
       </c>
@@ -3323,10 +3323,10 @@
         <v>17</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>108</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" s="2">
         <v>18</v>
       </c>
@@ -3334,10 +3334,10 @@
         <v>18</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>109</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" s="2">
         <v>19</v>
       </c>
@@ -3345,10 +3345,10 @@
         <v>14</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" s="2">
         <v>20</v>
       </c>
@@ -3356,10 +3356,10 @@
         <v>14</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" s="2">
         <v>21</v>
       </c>
@@ -3367,10 +3367,10 @@
         <v>14</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" s="2">
         <v>22</v>
       </c>
@@ -3378,10 +3378,10 @@
         <v>14</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25" s="2">
         <v>23</v>
       </c>
@@ -3389,10 +3389,10 @@
         <v>16</v>
       </c>
       <c r="C25" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" s="2">
         <v>24</v>
       </c>
@@ -3400,10 +3400,10 @@
         <v>16</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A27" s="2">
         <v>25</v>
       </c>
@@ -3411,10 +3411,10 @@
         <v>17</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" s="2">
         <v>26</v>
       </c>
@@ -3422,10 +3422,10 @@
         <v>17</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" s="2">
         <v>27</v>
       </c>
@@ -3433,10 +3433,10 @@
         <v>17</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" s="2">
         <v>28</v>
       </c>
@@ -3444,10 +3444,10 @@
         <v>18</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A31" s="2">
         <v>29</v>
       </c>
@@ -3455,10 +3455,10 @@
         <v>18</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A32" s="2">
         <v>30</v>
       </c>
@@ -3466,10 +3466,10 @@
         <v>19</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="2">
         <v>31</v>
       </c>
@@ -3477,10 +3477,10 @@
         <v>19</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="2">
         <v>32</v>
       </c>
@@ -3488,10 +3488,10 @@
         <v>22</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="2">
         <v>33</v>
       </c>
@@ -3499,11 +3499,11 @@
         <v>22</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="I35" s="5"/>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+        <v>25</v>
+      </c>
+      <c r="I35" s="3"/>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="2">
         <v>34</v>
       </c>
@@ -3511,10 +3511,10 @@
         <v>23</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="2">
         <v>35</v>
       </c>
@@ -3522,10 +3522,10 @@
         <v>25</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="2">
         <v>36</v>
       </c>
@@ -3533,10 +3533,10 @@
         <v>25</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="2">
         <v>37</v>
       </c>
@@ -3544,10 +3544,10 @@
         <v>25</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A40" s="2">
         <v>38</v>
       </c>
@@ -3555,10 +3555,10 @@
         <v>26</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" s="2">
         <v>39</v>
       </c>
@@ -3566,10 +3566,10 @@
         <v>26</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" s="2">
         <v>40</v>
       </c>
@@ -3577,10 +3577,10 @@
         <v>26</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" s="2">
         <v>41</v>
       </c>
@@ -3588,10 +3588,10 @@
         <v>29</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" s="2">
         <v>42</v>
       </c>
@@ -3599,10 +3599,10 @@
         <v>29</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" s="2">
         <v>43</v>
       </c>
@@ -3610,10 +3610,10 @@
         <v>29</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" s="2">
         <v>44</v>
       </c>
@@ -3621,10 +3621,10 @@
         <v>30</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A47" s="2">
         <v>45</v>
       </c>
@@ -3632,10 +3632,10 @@
         <v>30</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" s="2">
         <v>46</v>
       </c>
@@ -3643,10 +3643,10 @@
         <v>30</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A49" s="2">
         <v>47</v>
       </c>
@@ -3654,10 +3654,10 @@
         <v>30</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A50" s="2">
         <v>48</v>
       </c>
@@ -3665,10 +3665,10 @@
         <v>31</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A51" s="2">
         <v>49</v>
       </c>
@@ -3676,10 +3676,10 @@
         <v>32</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A52" s="2">
         <v>50</v>
       </c>
@@ -3687,10 +3687,10 @@
         <v>33</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A53" s="2">
         <v>51</v>
       </c>
@@ -3698,10 +3698,10 @@
         <v>33</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A54" s="2">
         <v>52</v>
       </c>
@@ -3709,10 +3709,10 @@
         <v>33</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>37</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A55" s="2">
         <v>53</v>
       </c>
@@ -3720,10 +3720,10 @@
         <v>33</v>
       </c>
       <c r="C55" s="2" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A56" s="2">
         <v>54</v>
       </c>
@@ -3731,10 +3731,10 @@
         <v>34</v>
       </c>
       <c r="C56" s="2" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A57" s="2">
         <v>55</v>
       </c>
@@ -3742,10 +3742,10 @@
         <v>34</v>
       </c>
       <c r="C57" s="2" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A58" s="2">
         <v>56</v>
       </c>
@@ -3753,10 +3753,10 @@
         <v>36</v>
       </c>
       <c r="C58" s="2" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A59" s="2">
         <v>57</v>
       </c>
@@ -3764,10 +3764,10 @@
         <v>36</v>
       </c>
       <c r="C59" s="2" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+        <v>150</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A60" s="2">
         <v>58</v>
       </c>
@@ -3775,10 +3775,10 @@
         <v>37</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A61" s="2">
         <v>59</v>
       </c>
@@ -3786,7 +3786,7 @@
         <v>37</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>